<commit_message>
Enhanced anchored index builder with formula extraction, cell references, chunk overlap, and environment variable configuration
</commit_message>
<xml_diff>
--- a/vansh-test/test.xlsx
+++ b/vansh-test/test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vansh/Documents/Documents/PROJECTS/skopeo-context/context-engine/vansh-test/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFFCB544-07D7-E248-B87A-417D55558900}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C72E5D06-8E10-284B-BF1D-7074F1909B40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4420" yWindow="680" windowWidth="15960" windowHeight="17880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4420" yWindow="680" windowWidth="15960" windowHeight="17840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Export Summary" sheetId="1" r:id="rId1"/>
@@ -4096,7 +4096,10 @@
         <v>17</v>
       </c>
       <c r="D4" s="17"/>
-      <c r="E4" s="12"/>
+      <c r="E4" s="12">
+        <f>SUM(D28:D31)</f>
+        <v>6071</v>
+      </c>
       <c r="F4" s="8"/>
       <c r="G4" s="9"/>
       <c r="H4" s="9"/>

</xml_diff>